<commit_message>
admission module with many issues_02
</commit_message>
<xml_diff>
--- a/Develpers_arp/EXCEL PLAN .xlsx
+++ b/Develpers_arp/EXCEL PLAN .xlsx
@@ -88,6 +88,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -153,12 +154,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -288,66 +293,66 @@
   <dimension ref="A1:S4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5.19"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="5.19"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="2" customFormat="true" ht="17.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="0"/>
-      <c r="S1" s="0"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>17</v>
       </c>
     </row>

</xml_diff>